<commit_message>
fix: correct known drug counts to unique drug_common_name, update ST1 caption
- Recomputed Known Drugs (DB) using unique drug_common_name per disease_id
  from Open Targets parquet (e.g., RA 2397→240, MS 1885→145)
- Preserved pipeline-derived Available/Recovered counts from git
- Updated Table1_Disease_Summary.csv with corrected counts and recovery rates
- Simplified ST1 caption (removed merge/colitis notes)
- Regenerated all autoimmune case study figures with corrected data
</commit_message>
<xml_diff>
--- a/autoimmune/analysis/recovery_summary/20_autoimmune.xlsx
+++ b/autoimmune/analysis/recovery_summary/20_autoimmune.xlsx
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>224</v>
+        <v>18</v>
       </c>
       <c r="D2" t="n">
         <v>978</v>
@@ -561,7 +561,7 @@
         <v>3</v>
       </c>
       <c r="P2" t="n">
-        <v>0.003067484662576687</v>
+        <v>0.1666666666666667</v>
       </c>
     </row>
     <row r="3">
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>605</v>
+        <v>53</v>
       </c>
       <c r="D3" t="n">
         <v>474</v>
@@ -615,7 +615,7 @@
         <v>13</v>
       </c>
       <c r="P3" t="n">
-        <v>0.02742616033755274</v>
+        <v>0.2452830188679245</v>
       </c>
     </row>
     <row r="4">
@@ -630,7 +630,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D4" t="n">
         <v>574</v>
@@ -669,7 +669,7 @@
         <v>25</v>
       </c>
       <c r="P4" t="n">
-        <v>0.04355400696864112</v>
+        <v>0.1677852348993289</v>
       </c>
     </row>
     <row r="5">
@@ -684,7 +684,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>630</v>
+        <v>47</v>
       </c>
       <c r="D5" t="n">
         <v>709</v>
@@ -723,7 +723,7 @@
         <v>6</v>
       </c>
       <c r="P5" t="n">
-        <v>0.008462623413258111</v>
+        <v>0.1276595744680851</v>
       </c>
     </row>
     <row r="6">
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>69</v>
+        <v>8</v>
       </c>
       <c r="D6" t="n">
         <v>419</v>
@@ -777,7 +777,7 @@
         <v>1</v>
       </c>
       <c r="P6" t="n">
-        <v>0.002386634844868735</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="7">
@@ -792,7 +792,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>84</v>
+        <v>9</v>
       </c>
       <c r="D7" t="n">
         <v>433</v>
@@ -831,7 +831,7 @@
         <v>2</v>
       </c>
       <c r="P7" t="n">
-        <v>0.004618937644341801</v>
+        <v>0.2222222222222222</v>
       </c>
     </row>
     <row r="8">
@@ -885,7 +885,7 @@
         <v>2</v>
       </c>
       <c r="P8" t="n">
-        <v>0.004319654427645789</v>
+        <v>0.06896551724137931</v>
       </c>
     </row>
     <row r="9">
@@ -900,7 +900,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>304</v>
+        <v>39</v>
       </c>
       <c r="D9" t="n">
         <v>1086</v>
@@ -939,7 +939,7 @@
         <v>8</v>
       </c>
       <c r="P9" t="n">
-        <v>0.007366482504604052</v>
+        <v>0.2051282051282051</v>
       </c>
     </row>
     <row r="10">
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>538</v>
+        <v>33</v>
       </c>
       <c r="D10" t="n">
         <v>503</v>
@@ -993,7 +993,7 @@
         <v>6</v>
       </c>
       <c r="P10" t="n">
-        <v>0.01192842942345924</v>
+        <v>0.1818181818181818</v>
       </c>
     </row>
     <row r="11">
@@ -1008,7 +1008,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>634</v>
+        <v>43</v>
       </c>
       <c r="D11" t="n">
         <v>417</v>
@@ -1047,7 +1047,7 @@
         <v>7</v>
       </c>
       <c r="P11" t="n">
-        <v>0.01678657074340528</v>
+        <v>0.1627906976744186</v>
       </c>
     </row>
     <row r="12">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1283</v>
+        <v>104</v>
       </c>
       <c r="D12" t="n">
         <v>476</v>
@@ -1101,7 +1101,7 @@
         <v>11</v>
       </c>
       <c r="P12" t="n">
-        <v>0.02310924369747899</v>
+        <v>0.1057692307692308</v>
       </c>
     </row>
     <row r="13">
@@ -1116,7 +1116,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>816</v>
+        <v>79</v>
       </c>
       <c r="D13" t="n">
         <v>1065</v>
@@ -1155,7 +1155,7 @@
         <v>12</v>
       </c>
       <c r="P13" t="n">
-        <v>0.01126760563380282</v>
+        <v>0.1518987341772152</v>
       </c>
     </row>
     <row r="14">
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2397</v>
+        <v>240</v>
       </c>
       <c r="D14" t="n">
         <v>859</v>
@@ -1209,7 +1209,7 @@
         <v>22</v>
       </c>
       <c r="P14" t="n">
-        <v>0.02561117578579744</v>
+        <v>0.09166666666666666</v>
       </c>
     </row>
     <row r="15">
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1071</v>
+        <v>103</v>
       </c>
       <c r="D15" t="n">
         <v>894</v>
@@ -1263,7 +1263,7 @@
         <v>16</v>
       </c>
       <c r="P15" t="n">
-        <v>0.01789709172259508</v>
+        <v>0.1553398058252427</v>
       </c>
     </row>
     <row r="16">
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1192</v>
+        <v>115</v>
       </c>
       <c r="D16" t="n">
         <v>619</v>
@@ -1317,7 +1317,7 @@
         <v>8</v>
       </c>
       <c r="P16" t="n">
-        <v>0.01292407108239095</v>
+        <v>0.06956521739130435</v>
       </c>
     </row>
     <row r="17">
@@ -1332,7 +1332,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1885</v>
+        <v>145</v>
       </c>
       <c r="D17" t="n">
         <v>774</v>
@@ -1371,7 +1371,7 @@
         <v>18</v>
       </c>
       <c r="P17" t="n">
-        <v>0.02325581395348837</v>
+        <v>0.1241379310344828</v>
       </c>
     </row>
     <row r="18">
@@ -1386,7 +1386,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="D18" t="n">
         <v>191</v>
@@ -1425,7 +1425,7 @@
         <v>3</v>
       </c>
       <c r="P18" t="n">
-        <v>0.01570680628272251</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="19">
@@ -1440,7 +1440,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1788</v>
+        <v>138</v>
       </c>
       <c r="D19" t="n">
         <v>807</v>
@@ -1479,7 +1479,7 @@
         <v>10</v>
       </c>
       <c r="P19" t="n">
-        <v>0.01239157372986369</v>
+        <v>0.07246376811594203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>